<commit_message>
UDF (fonctions de feuille) + menu ruban "UDF Sync"
- Functions.cs : UDF [ExcelFunction] POC.ADDITION, POC.BONJOUR + UDF a plage
  (object[,]/double[,]/object[]) SOMMEPERSO, CONCAT, MOYENNE, COMPTENB,
  INFOPLAGE, PRODUITSCALAIRE (2 plages), DOUBLER (renvoie un tableau).
- RibbonController.Udf.cs : menu "UDF Sync" ; chaque entree insere un exemple
  pret a l emploi (constantes matricielles) dans la selection via .Formula
  (formule portee par le tag du bouton, un seul callback OnInsertFormula).
- TestAddin.xlsx : feuille "UDF" avec exemples 1D et 2D (A2:B5).
- .gitignore : ignore les copies de conflit OneDrive.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TestAddin.xlsx
+++ b/TestAddin.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c2c05a52312f03d6/Documents/GitHub/ExcelDnaPoc/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\romai\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{428C5F1A-D8E3-4766-95E8-33BF32E34E2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0494B966-A480-455A-AD15-89DE4DB7A940}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{41D53E50-B3EF-478D-B03E-D92CA89DF6CF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{F8782059-B33D-4519-BF89-B20E33AAF9E3}"/>
   </bookViews>
   <sheets>
     <sheet name="TestAddin" sheetId="1" r:id="rId1"/>
+    <sheet name="UDF" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>BlagueMenuExcel</t>
   </si>
@@ -48,6 +49,63 @@
   </si>
   <si>
     <t>BlagueMenuWpf</t>
+  </si>
+  <si>
+    <t>Donnees</t>
+  </si>
+  <si>
+    <t>(num)</t>
+  </si>
+  <si>
+    <t>texte</t>
+  </si>
+  <si>
+    <t>Plages 1D (colonne)</t>
+  </si>
+  <si>
+    <t>Resultat</t>
+  </si>
+  <si>
+    <t>POC.ADDITION(2;3)</t>
+  </si>
+  <si>
+    <t>POC.BONJOUR("Romain")</t>
+  </si>
+  <si>
+    <t>POC.SOMMEPERSO(A2:A5)</t>
+  </si>
+  <si>
+    <t>POC.CONCAT(A2:A5;" | ")</t>
+  </si>
+  <si>
+    <t>POC.MOYENNE(B2:B5)</t>
+  </si>
+  <si>
+    <t>POC.COMPTENB(A2:A5)</t>
+  </si>
+  <si>
+    <t>POC.INFOPLAGE(A2:A5)</t>
+  </si>
+  <si>
+    <t>POC.PRODUITSCALAIRE(B2:B5;B2:B5)</t>
+  </si>
+  <si>
+    <t>Plages 2D (A2:B5 = 4 lignes x 2 colonnes)</t>
+  </si>
+  <si>
+    <t>POC.SOMMEPERSO(A2:B5)</t>
+  </si>
+  <si>
+    <t>POC.INFOPLAGE(A2:B5)</t>
+  </si>
+  <si>
+    <t>POC.CONCAT(A2:B5;" | ")</t>
+  </si>
+  <si>
+    <t>POC.DOUBLER(A2:B5) -&gt; G2:H5 (matricielle 4x2)</t>
+  </si>
+  <si>
+    <t>DOUBLER(A2:B5)</t>
   </si>
 </sst>
 </file>
@@ -418,7 +476,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC86F8AA-EC92-4CF2-B2D0-A312016F0AC0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2174331A-D0C8-4DDF-B2D1-38C339B00919}">
   <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -440,4 +498,193 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{975A8D7A-643D-4E35-BD52-BBC7E1ECD814}">
+  <dimension ref="A1:H16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="4" max="4" width="40.77734375" customWidth="1"/>
+    <col min="5" max="5" width="34.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>10</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2">
+        <f>_xll.POC.ADDITION(2,3)</f>
+        <v>5</v>
+      </c>
+      <c r="G2">
+        <f t="array" ref="G2:H5">_xll.POC.DOUBLER(A2:B5)</f>
+        <v>20</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>20</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" t="str">
+        <f>_xll.POC.BONJOUR("Romain")</f>
+        <v>Bonjour Romain !</v>
+      </c>
+      <c r="G3">
+        <v>40</v>
+      </c>
+      <c r="H3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4">
+        <f>_xll.POC.SOMMEPERSO(A2:A5)</f>
+        <v>35</v>
+      </c>
+      <c r="G4" t="str">
+        <v>texte</v>
+      </c>
+      <c r="H4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="str">
+        <f>_xll.POC.CONCAT(A2:A5," | ")</f>
+        <v>10 | 20 | texte | 5</v>
+      </c>
+      <c r="G5">
+        <v>10</v>
+      </c>
+      <c r="H5">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6">
+        <f>_xll.POC.MOYENNE(B2:B5)</f>
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7">
+        <f>_xll.POC.COMPTENB(A2:A5)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" t="str">
+        <f>_xll.POC.INFOPLAGE(A2:A5)</f>
+        <v>3 nombre(s), 1 texte(s), 0 vide(s), 0 erreur(s)</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9">
+        <f>_xll.POC.PRODUITSCALAIRE(B2:B5,B2:B5)</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D12" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D13" t="s">
+        <v>17</v>
+      </c>
+      <c r="E13">
+        <f>_xll.POC.SOMMEPERSO(A2:B5)</f>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D14" t="s">
+        <v>18</v>
+      </c>
+      <c r="E14" t="str">
+        <f>_xll.POC.INFOPLAGE(A2:B5)</f>
+        <v>7 nombre(s), 1 texte(s), 0 vide(s), 0 erreur(s)</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E15" t="str">
+        <f>_xll.POC.CONCAT(A2:B5," | ")</f>
+        <v>10 | 1 | 20 | 2 | texte | 3 | 5 | 4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D16" t="s">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>